<commit_message>
figma prototye and revised required doc file
</commit_message>
<xml_diff>
--- a/Week_5/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_5/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
   <si>
     <t>Week_1</t>
   </si>
@@ -155,6 +155,12 @@
   </si>
   <si>
     <t>Wireframe in Figma Prototyping) (Public Pages)</t>
+  </si>
+  <si>
+    <t>Wire frame Prototyping (All pages)</t>
+  </si>
+  <si>
+    <t>Revised Requirment document file</t>
   </si>
 </sst>
 </file>
@@ -2665,9 +2671,15 @@
     </row>
     <row r="60">
       <c r="A60" s="41"/>
-      <c r="B60" s="42"/>
-      <c r="C60" s="43"/>
-      <c r="D60" s="44"/>
+      <c r="B60" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="C60" s="43">
+        <v>46069.0</v>
+      </c>
+      <c r="D60" s="44">
+        <v>3.5</v>
+      </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -2694,9 +2706,15 @@
     </row>
     <row r="61">
       <c r="A61" s="41"/>
-      <c r="B61" s="42"/>
-      <c r="C61" s="43"/>
-      <c r="D61" s="44"/>
+      <c r="B61" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="C61" s="43">
+        <v>46069.0</v>
+      </c>
+      <c r="D61" s="44">
+        <v>2.5</v>
+      </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -2787,7 +2805,7 @@
       <c r="C64" s="47"/>
       <c r="D64" s="41">
         <f>sum(D58:D62)</f>
-        <v>5.9</v>
+        <v>11.9</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>

</xml_diff>